<commit_message>
v5.0: python_regel gevuld voor 11 deterministische AP's (briefing §3, 13 okt)
Notatie <grootheid> <op> <waarde>, ' en ' / ' of '. Leeg bij alle andere AP's.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/261013_Prompts_aandachtspunten_v5.0.xlsx
+++ b/261013_Prompts_aandachtspunten_v5.0.xlsx
@@ -590,12 +590,12 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Zoek naar / Blokken / Python-regel</t>
+          <t>Python-regel</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Blijven staan maar worden door de code niet (meer) gebruikt (briefing §3).</t>
+          <t>Gevuld voor 11 deterministische AP's in de notatie uit briefing §3 (`&lt;grootheid&gt; &lt;op&gt; &lt;waarde&gt;`, ` en ` / ` of `). Leeg bij alle andere. `zoek_naar` en `blokken` blijven staan maar worden niet gebruikt.</t>
         </is>
       </c>
     </row>
@@ -1522,7 +1522,11 @@
         </is>
       </c>
       <c r="K11" s="9" t="inlineStr"/>
-      <c r="L11" s="8" t="inlineStr"/>
+      <c r="L11" s="8" t="inlineStr">
+        <is>
+          <t>bmi &gt;= 30 en &lt; 35</t>
+        </is>
+      </c>
       <c r="M11" s="7" t="inlineStr">
         <is>
           <t>Gezamenlijk BMI-meetmoment voor AP010–AP012/AP044 en omgang met alleen een zorgpadvermelding.</t>
@@ -1543,7 +1547,7 @@
       </c>
       <c r="S11" s="8" t="inlineStr">
         <is>
-          <t>Getallen expliciet; periode (intake) expliciet.</t>
+          <t>Getallen expliciet; periode (intake) expliciet. python_regel: `bmi &gt;= 30 en &lt; 35` (briefing §3).</t>
         </is>
       </c>
     </row>
@@ -1599,7 +1603,11 @@
         </is>
       </c>
       <c r="K12" s="9" t="inlineStr"/>
-      <c r="L12" s="8" t="inlineStr"/>
+      <c r="L12" s="8" t="inlineStr">
+        <is>
+          <t>bmi &gt;= 35 en &lt; 40</t>
+        </is>
+      </c>
       <c r="M12" s="7" t="inlineStr"/>
       <c r="N12" s="7" t="inlineStr"/>
       <c r="O12" s="8" t="inlineStr"/>
@@ -1616,7 +1624,7 @@
       </c>
       <c r="S12" s="8" t="inlineStr">
         <is>
-          <t>Zie AP010.</t>
+          <t>Zie AP010. python_regel: `bmi &gt;= 35 en &lt; 40` (briefing §3).</t>
         </is>
       </c>
     </row>
@@ -1672,7 +1680,11 @@
         </is>
       </c>
       <c r="K13" s="9" t="inlineStr"/>
-      <c r="L13" s="8" t="inlineStr"/>
+      <c r="L13" s="8" t="inlineStr">
+        <is>
+          <t>bmi &gt;= 40</t>
+        </is>
+      </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
           <t>Het oorspronkelijke label was ‘&gt;40’. Voor een aaneensluitende indeling is dit gewijzigd naar ‘≥40’; laat deze wijziging bevestigen. De bariatrische subcategorieën houden voorlopig hun oorspronkelijke indeling aan.</t>
@@ -1693,7 +1705,7 @@
       </c>
       <c r="S13" s="8" t="inlineStr">
         <is>
-          <t>Zie AP010.</t>
+          <t>Zie AP010. python_regel: `bmi &gt;= 40` (briefing §3).</t>
         </is>
       </c>
     </row>
@@ -2949,7 +2961,11 @@
         </is>
       </c>
       <c r="K30" s="9" t="inlineStr"/>
-      <c r="L30" s="8" t="inlineStr"/>
+      <c r="L30" s="8" t="inlineStr">
+        <is>
+          <t>hbsag == positief</t>
+        </is>
+      </c>
       <c r="M30" s="7" t="inlineStr"/>
       <c r="N30" s="7" t="inlineStr"/>
       <c r="O30" s="8" t="inlineStr"/>
@@ -2966,7 +2982,7 @@
       </c>
       <c r="S30" s="8" t="inlineStr">
         <is>
-          <t>Negatieve uitslag en familie als ontkenning expliciet.</t>
+          <t>Negatieve uitslag en familie als ontkenning expliciet. python_regel: `hbsag == positief` (briefing §3).</t>
         </is>
       </c>
     </row>
@@ -3095,7 +3111,11 @@
         </is>
       </c>
       <c r="K32" s="9" t="inlineStr"/>
-      <c r="L32" s="8" t="inlineStr"/>
+      <c r="L32" s="8" t="inlineStr">
+        <is>
+          <t>hiv == positief</t>
+        </is>
+      </c>
       <c r="M32" s="7" t="inlineStr"/>
       <c r="N32" s="7" t="inlineStr"/>
       <c r="O32" s="8" t="inlineStr"/>
@@ -3112,7 +3132,7 @@
       </c>
       <c r="S32" s="8" t="inlineStr">
         <is>
-          <t>Negatieve test en partner als ontkenning.</t>
+          <t>Negatieve test en partner als ontkenning. python_regel: `hiv == positief` (briefing §3).</t>
         </is>
       </c>
     </row>
@@ -4068,7 +4088,11 @@
         </is>
       </c>
       <c r="K45" s="9" t="inlineStr"/>
-      <c r="L45" s="8" t="inlineStr"/>
+      <c r="L45" s="8" t="inlineStr">
+        <is>
+          <t>bmi &lt; 18.5</t>
+        </is>
+      </c>
       <c r="M45" s="7" t="inlineStr"/>
       <c r="N45" s="7" t="inlineStr"/>
       <c r="O45" s="8" t="inlineStr"/>
@@ -4085,7 +4109,7 @@
       </c>
       <c r="S45" s="8" t="inlineStr">
         <is>
-          <t>Getal expliciet (het gemelde 18,69-geval).</t>
+          <t>Getal expliciet (het gemelde 18,69-geval). python_regel: `bmi &lt; 18.5` (briefing §3).</t>
         </is>
       </c>
     </row>
@@ -4441,7 +4465,11 @@
         </is>
       </c>
       <c r="K50" s="9" t="inlineStr"/>
-      <c r="L50" s="8" t="inlineStr"/>
+      <c r="L50" s="8" t="inlineStr">
+        <is>
+          <t>leeftijd &gt;= 40</t>
+        </is>
+      </c>
       <c r="M50" s="7" t="inlineStr"/>
       <c r="N50" s="7" t="inlineStr"/>
       <c r="O50" s="8" t="inlineStr"/>
@@ -4458,7 +4486,7 @@
       </c>
       <c r="S50" s="8" t="inlineStr">
         <is>
-          <t>Getal en referentiedatum expliciet.</t>
+          <t>Getal en referentiedatum expliciet. python_regel: `leeftijd &gt;= 40` (briefing §3).</t>
         </is>
       </c>
     </row>
@@ -4980,7 +5008,11 @@
         </is>
       </c>
       <c r="K57" s="9" t="inlineStr"/>
-      <c r="L57" s="8" t="inlineStr"/>
+      <c r="L57" s="8" t="inlineStr">
+        <is>
+          <t>hb &lt; 7.1 of ferritine &lt; 15</t>
+        </is>
+      </c>
       <c r="M57" s="7" t="inlineStr">
         <is>
           <t>Of een expliciete diagnose zonder meetwaarden zelfstandig mag meetellen. De numerieke grenzen en uitsluiting van suppletie zijn definitief afgesproken; dit diagnose-alternatief is een conceptregel voor kaarten met ontbrekende waarden.</t>
@@ -5001,7 +5033,7 @@
       </c>
       <c r="S57" s="8" t="inlineStr">
         <is>
-          <t>Periode (huidig; geen Hb van na een vorige bevalling) en normale waarde expliciet.</t>
+          <t>Periode (huidig; geen Hb van na een vorige bevalling) en normale waarde expliciet. python_regel: `hb &lt; 7.1 of ferritine &lt; 15` (briefing §3).</t>
         </is>
       </c>
     </row>
@@ -5057,7 +5089,11 @@
         </is>
       </c>
       <c r="K58" s="9" t="inlineStr"/>
-      <c r="L58" s="8" t="inlineStr"/>
+      <c r="L58" s="8" t="inlineStr">
+        <is>
+          <t>rhesus_d == negatief</t>
+        </is>
+      </c>
       <c r="M58" s="7" t="inlineStr"/>
       <c r="N58" s="7" t="inlineStr"/>
       <c r="O58" s="8" t="inlineStr"/>
@@ -5074,7 +5110,7 @@
       </c>
       <c r="S58" s="8" t="inlineStr">
         <is>
-          <t>'O pos' expliciet niet positief.</t>
+          <t>'O pos' expliciet niet positief. python_regel: `rhesus_d == negatief` (briefing §3).</t>
         </is>
       </c>
     </row>
@@ -5130,7 +5166,11 @@
         </is>
       </c>
       <c r="K59" s="9" t="inlineStr"/>
-      <c r="L59" s="8" t="inlineStr"/>
+      <c r="L59" s="8" t="inlineStr">
+        <is>
+          <t>rhesus_c == negatief</t>
+        </is>
+      </c>
       <c r="M59" s="7" t="inlineStr"/>
       <c r="N59" s="7" t="inlineStr"/>
       <c r="O59" s="8" t="inlineStr"/>
@@ -5147,7 +5187,7 @@
       </c>
       <c r="S59" s="8" t="inlineStr">
         <is>
-          <t>Ingekort; D-status als ontkenning.</t>
+          <t>Ingekort; D-status als ontkenning. python_regel: `rhesus_c == negatief` (briefing §3).</t>
         </is>
       </c>
     </row>
@@ -6192,7 +6232,11 @@
         </is>
       </c>
       <c r="K73" s="9" t="inlineStr"/>
-      <c r="L73" s="8" t="inlineStr"/>
+      <c r="L73" s="8" t="inlineStr">
+        <is>
+          <t>trombocyten &lt; 150</t>
+        </is>
+      </c>
       <c r="M73" s="7" t="inlineStr"/>
       <c r="N73" s="7" t="inlineStr"/>
       <c r="O73" s="8" t="inlineStr"/>
@@ -6209,7 +6253,7 @@
       </c>
       <c r="S73" s="8" t="inlineStr">
         <is>
-          <t>Getal en periode expliciet.</t>
+          <t>Getal en periode expliciet. python_regel: `trombocyten &lt; 150` (briefing §3).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v5.0: AP004-006/AP070 formulering twee voorwaarden (bouwer), AP059 python_regel interval_maanden < 12
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/261013_Prompts_aandachtspunten_v5.0.xlsx
+++ b/261013_Prompts_aandachtspunten_v5.0.xlsx
@@ -1052,12 +1052,12 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>De passage noemt een uitgevoerde bariatrische ingreep (gastric bypass, sleeve, maagband, maagverkleining, WLS) bij de zwangere; de BMI 30–40 is een tweede voorwaarde die de zorgverlener met de BMI-vermelding combineert.</t>
+          <t>Een doorgemaakte bariatrische operatie (gastric bypass, sleeve, maagband, maagverkleining, WLS) bij de zwangere is vermeld. Een BMI-waarde alleen, zonder operatie, is niet positief; de BMI-grens (30 tot 40) combineert de zorgverlener.</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>Een BMI-, lengte- of gewichtsvermelding zonder operatie is nooit positief; alleen obesitas, dumping, suppletie of een geplande ingreep; een BMI buiten 30–40.</t>
+          <t>Een BMI-, lengte- of gewichtsvermelding zonder operatie; alleen obesitas, dumping, suppletie of een geplande ingreep; een BMI buiten 30–40.</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr">
@@ -1097,7 +1097,7 @@
       </c>
       <c r="S5" s="8" t="inlineStr">
         <is>
-          <t>Geen halve treffers: BMI alleen is nooit positief; operatie is de kernvoorwaarde.</t>
+          <t>Geen halve treffers: BMI alleen is nooit positief; operatie is de kernvoorwaarde. Formulering twee voorwaarden overgenomen van de bouwer (13-10): operatiepassage ja, BMI alleen nee.</t>
         </is>
       </c>
     </row>
@@ -1129,12 +1129,12 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>De passage noemt een uitgevoerde bariatrische ingreep (gastric bypass, sleeve, maagband, maagverkleining, WLS) bij de zwangere; de BMI ≥40 is een tweede voorwaarde die de zorgverlener met de BMI-vermelding combineert.</t>
+          <t>Een doorgemaakte bariatrische operatie (gastric bypass, sleeve, maagband, maagverkleining, WLS) bij de zwangere is vermeld. Een BMI-waarde alleen, zonder operatie, is niet positief; de BMI-grens (≥40) combineert de zorgverlener.</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>Een BMI-, lengte- of gewichtsvermelding zonder operatie is nooit positief; alleen morbide obesitas of een geplande ingreep; een BMI &lt;40.</t>
+          <t>Een BMI-, lengte- of gewichtsvermelding zonder operatie; alleen morbide obesitas of een geplande ingreep; een BMI &lt;40.</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
@@ -1170,7 +1170,7 @@
       </c>
       <c r="S6" s="8" t="inlineStr">
         <is>
-          <t>Zie AP004.</t>
+          <t>Zie AP004. Formulering twee voorwaarden overgenomen van de bouwer (13-10): operatiepassage ja, BMI alleen nee.</t>
         </is>
       </c>
     </row>
@@ -1202,12 +1202,12 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>De passage noemt een uitgevoerde bariatrische ingreep (gastric bypass, sleeve, maagband, maagverkleining, WLS) bij de zwangere; de BMI &lt;30 is een tweede voorwaarde die de zorgverlener met de BMI-vermelding combineert.</t>
+          <t>Een doorgemaakte bariatrische operatie (gastric bypass, sleeve, maagband, maagverkleining, WLS) bij de zwangere is vermeld. Een BMI-waarde alleen, zonder operatie, is niet positief; de BMI-grens (&lt;30) combineert de zorgverlener.</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>Een BMI-, lengte- of gewichtsvermelding zonder operatie is nooit positief; alleen suppletie, dagcurve of een geplande ingreep; een BMI ≥30.</t>
+          <t>Een BMI-, lengte- of gewichtsvermelding zonder operatie; alleen suppletie, dagcurve of een geplande ingreep; een BMI ≥30.</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
@@ -1243,7 +1243,7 @@
       </c>
       <c r="S7" s="8" t="inlineStr">
         <is>
-          <t>Zie AP004 (dit was het gemelde geval 'BMI 23.7' zonder operatie).</t>
+          <t>Zie AP004 (dit was het gemelde geval 'BMI 23.7' zonder operatie). Formulering twee voorwaarden overgenomen van de bouwer (13-10): operatiepassage ja, BMI alleen nee.</t>
         </is>
       </c>
     </row>
@@ -5243,7 +5243,11 @@
         </is>
       </c>
       <c r="K60" s="9" t="inlineStr"/>
-      <c r="L60" s="8" t="inlineStr"/>
+      <c r="L60" s="8" t="inlineStr">
+        <is>
+          <t>interval_maanden &lt; 12</t>
+        </is>
+      </c>
       <c r="M60" s="7" t="inlineStr"/>
       <c r="N60" s="7" t="inlineStr"/>
       <c r="O60" s="8" t="inlineStr"/>
@@ -5260,7 +5264,7 @@
       </c>
       <c r="S60" s="8" t="inlineStr">
         <is>
-          <t>Geformuleerd met datums (AD − 266 dagen); grootste ruisbron.</t>
+          <t>Geformuleerd met datums (AD − 266 dagen); grootste ruisbron. python_regel `interval_maanden &lt; 12` (grootheid bouwt de bouwer; betekenis blijft voor onbepaalde datums).</t>
         </is>
       </c>
     </row>
@@ -6054,12 +6058,12 @@
       </c>
       <c r="F71" s="7" t="inlineStr">
         <is>
-          <t>De passage noemt in deze zwangerschap een velamenteuze (vliezige) insertie van de navelstreng; 'vasa praevia uitgesloten' is een tweede voorwaarde die de zorgverlener combineert.</t>
+          <t>Een velamenteuze (vliezige) insertie van de navelstreng in deze zwangerschap is vermeld. Een vermelding over vasa praevia alleen is niet positief; of vasa praevia is uitgesloten combineert de zorgverlener.</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
         <is>
-          <t>Een marginale of ongespecificeerde insertie; vasa praevia zelf; een normale insertie; 'vasa praevia nog uit te sluiten' zonder velamenteuze insertie.</t>
+          <t>Een marginale of ongespecificeerde insertie; vasa praevia zonder velamenteuze insertie; een normale insertie.</t>
         </is>
       </c>
       <c r="H71" s="7" t="inlineStr">
@@ -6099,7 +6103,7 @@
       </c>
       <c r="S71" s="8" t="inlineStr">
         <is>
-          <t>Twee voorwaarden benoemd; ingekort.</t>
+          <t>Twee voorwaarden benoemd; ingekort. Zelfde aanpak als AP004–006: insertiepassage ja, vasa praevia alleen nee (13-10).</t>
         </is>
       </c>
     </row>

</xml_diff>